<commit_message>
deploy: update generated archive
</commit_message>
<xml_diff>
--- a/assets/books/academic-survival-manual-appendix-v3.1.xlsx
+++ b/assets/books/academic-survival-manual-appendix-v3.1.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 리젝션 48시간" sheetId="1" r:id="R8d057959863447e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 멘토 미팅 준비" sheetId="2" r:id="R90a6904428ae4c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 프로젝트 중단" sheetId="3" r:id="Re742ba3c665943be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 학회 선택" sheetId="4" r:id="R8466bd736cc7474a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 한 학기 종료 리뷰" sheetId="5" r:id="R9eac8d84f6b44420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 발표 질문 준비" sheetId="6" r:id="Rd6f009e60dd64625"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 첫해 교수 운영" sheetId="7" r:id="Rd3201ee6b9ec4f9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 진학 프로그램 비교" sheetId="8" r:id="R07bce2c90b8c4018"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 평가 일정 역산" sheetId="9" r:id="R54b664ae18764d46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 리젝션 48시간" sheetId="1" r:id="Rb18781b0808447cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 멘토 미팅 준비" sheetId="2" r:id="Rd80ff462e9b844db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 프로젝트 중단" sheetId="3" r:id="R76ac9c121ef349a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 학회 선택" sheetId="4" r:id="R98e47c01444d47bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 한 학기 종료 리뷰" sheetId="5" r:id="R12af9ffc8ce44cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 발표 질문 준비" sheetId="6" r:id="Re6003d49213c4036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 첫해 교수 운영" sheetId="7" r:id="R5d957335d0be4a36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 진학 프로그램 비교" sheetId="8" r:id="R0cfb4caa7625414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 평가 일정 역산" sheetId="9" r:id="R8dbc36a5f9fd439d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -771,12 +771,6 @@
       </x:c>
       <x:c r="B10" s="16" t="str"/>
     </x:row>
-    <x:row r="11" ht="44" customHeight="1">
-      <x:c r="A11" s="16" t="str">
-        <x:v>내가 던질 질문</x:v>
-      </x:c>
-      <x:c r="B11" s="16" t="str"/>
-    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:B1"/>
@@ -922,84 +916,84 @@
     </x:row>
     <x:row r="4" ht="44" customHeight="1">
       <x:c r="A4" s="16" t="str">
-        <x:v>재정 지원 보장 기간</x:v>
+        <x:v>지도교수 접근성과 학생 수</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str"/>
       <x:c r="C4" s="16" t="str"/>
     </x:row>
     <x:row r="5" ht="44" customHeight="1">
       <x:c r="A5" s="16" t="str">
-        <x:v>월 실수령 지원금</x:v>
+        <x:v>최근 졸업생 진로</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str"/>
       <x:c r="C5" s="16" t="str"/>
     </x:row>
     <x:row r="6" ht="44" customHeight="1">
       <x:c r="A6" s="16" t="str">
-        <x:v>등록금·수수료·건강보험</x:v>
+        <x:v>학계 밖 경험·인턴십 가능성</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str"/>
       <x:c r="C6" s="16" t="str"/>
     </x:row>
     <x:row r="7" ht="44" customHeight="1">
       <x:c r="A7" s="16" t="str">
-        <x:v>여름 지원</x:v>
+        <x:v>중도 이탈·전환 시 남는 선택지</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str"/>
       <x:c r="C7" s="16" t="str"/>
     </x:row>
     <x:row r="8" ht="44" customHeight="1">
       <x:c r="A8" s="16" t="str">
-        <x:v>평균 주거비와 통학 조건</x:v>
+        <x:v>국제학생 지원과 비자 경로</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str"/>
       <x:c r="C8" s="16" t="str"/>
     </x:row>
     <x:row r="9" ht="44" customHeight="1">
       <x:c r="A9" s="16" t="str">
-        <x:v>지도교수 접근성과 학생 수</x:v>
+        <x:v>내가 감당하기 어려운 조건</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str"/>
       <x:c r="C9" s="16" t="str"/>
     </x:row>
     <x:row r="10" ht="44" customHeight="1">
       <x:c r="A10" s="16" t="str">
-        <x:v>최근 졸업생 진로</x:v>
+        <x:v>다음 확인 질문과 담당자</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str"/>
       <x:c r="C10" s="16" t="str"/>
     </x:row>
     <x:row r="11" ht="44" customHeight="1">
       <x:c r="A11" s="16" t="str">
-        <x:v>중도 이탈·전환 시 남는 선택지</x:v>
+        <x:v>재정 지원 보장 기간</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str"/>
       <x:c r="C11" s="16" t="str"/>
     </x:row>
     <x:row r="12" ht="44" customHeight="1">
       <x:c r="A12" s="16" t="str">
-        <x:v>국제학생 지원과 비자 경로</x:v>
+        <x:v>월 실수령 지원금</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str"/>
       <x:c r="C12" s="16" t="str"/>
     </x:row>
     <x:row r="13" ht="44" customHeight="1">
       <x:c r="A13" s="16" t="str">
-        <x:v>학계 밖 경험·인턴십 가능성</x:v>
+        <x:v>등록금·수수료·건강보험</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str"/>
       <x:c r="C13" s="16" t="str"/>
     </x:row>
     <x:row r="14" ht="44" customHeight="1">
       <x:c r="A14" s="16" t="str">
-        <x:v>내가 감당하기 어려운 조건</x:v>
+        <x:v>여름 지원</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str"/>
       <x:c r="C14" s="16" t="str"/>
     </x:row>
     <x:row r="15" ht="44" customHeight="1">
       <x:c r="A15" s="16" t="str">
-        <x:v>다음 확인 질문과 담당자</x:v>
+        <x:v>평균 주거비와 통학 조건</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str"/>
       <x:c r="C15" s="16" t="str"/>

</xml_diff>